<commit_message>
update test cases sheet
</commit_message>
<xml_diff>
--- a/src/test/resources/TestCases.xlsx
+++ b/src/test/resources/TestCases.xlsx
@@ -9,14 +9,13 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
   <si>
     <t xml:space="preserve">I have lots of embeded files in me</t>
   </si>
@@ -33,10 +32,16 @@
     <t xml:space="preserve">APIs consumed for Accounts loading</t>
   </si>
   <si>
+    <t>/apis/accounts/web/getCASAAccounts/1.0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify unauthorized access of the cas</t>
+  </si>
+  <si>
     <t>Completed</t>
   </si>
   <si>
-    <t>/apis/accounts/web/getCASAAccounts/1.0.0</t>
+    <t xml:space="preserve">Verify retrive casssa details using valid details</t>
   </si>
   <si>
     <t>/apis/accounts/web/getFDAccounts/1.0.0</t>
@@ -144,7 +149,6 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color indexed="64"/>
         <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve">Mobile Cash Received List  - </t>
@@ -153,7 +157,6 @@
       <rPr>
         <u val="single"/>
         <sz val="11"/>
-        <color indexed="64"/>
         <rFont val="Calibri"/>
       </rPr>
       <t>/apis/transaction/web/getUnutilizedMobileCashByBeneID/1.0.0</t>
@@ -401,7 +404,6 @@
     </font>
     <font>
       <sz val="11.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -445,7 +447,6 @@
     </font>
     <font>
       <sz val="11.000000"/>
-      <color indexed="64"/>
       <name val="Symbol"/>
     </font>
     <font>
@@ -654,7 +655,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -784,6 +785,32 @@
       </bottom>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="48">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -835,7 +862,7 @@
     <xf fontId="17" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="18" fillId="33" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -850,26 +877,36 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="4" fillId="23" borderId="0" numFmtId="0" xfId="22" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="29" borderId="10" numFmtId="0" xfId="33" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="1" fillId="23" borderId="0" numFmtId="0" xfId="22" applyFont="1" applyFill="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="12" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="1" fillId="23" borderId="0" numFmtId="0" xfId="22" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="1" fillId="23" borderId="0" numFmtId="0" xfId="22" applyFont="1" applyFill="1"/>
     <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="6" fillId="29" borderId="10" numFmtId="0" xfId="33" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf fontId="4" fillId="23" borderId="0" numFmtId="0" xfId="22" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="6" fillId="29" borderId="0" numFmtId="0" xfId="33" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1662,665 +1699,801 @@
   <cols>
     <col min="1" max="1" style="0" width="9.140625"/>
     <col customWidth="1" min="2" max="2" style="1" width="89.8515625"/>
-    <col customWidth="1" min="3" max="3" style="2" width="20.28125"/>
-    <col customWidth="1" min="4" max="4" style="0" width="56.140625"/>
-    <col min="5" max="5" style="0" width="9.140625"/>
-    <col min="6" max="16384" style="0" width="9.140625"/>
+    <col customWidth="1" min="3" max="4" style="1" width="55.140625"/>
+    <col customWidth="1" min="5" max="5" style="2" width="20.28125"/>
+    <col customWidth="1" min="6" max="6" style="0" width="56.140625"/>
+    <col min="7" max="16384" style="0" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="27.75" customHeight="1">
-      <c r="A1"/>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
-      <c r="A2"/>
+    <row r="2" ht="22.5" customHeight="1">
       <c r="B2" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="7"/>
-    </row>
-    <row r="3" ht="15" customHeight="1">
-      <c r="A3"/>
-      <c r="B3" s="8" t="s">
+      <c r="D2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="10"/>
+      <c r="E2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="10"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="12"/>
+      <c r="F3" s="9"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4"/>
-      <c r="B4" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="10"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="13"/>
+      <c r="E4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="14"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5"/>
-      <c r="B5" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" s="10"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="13"/>
+      <c r="E5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="14"/>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="B6" s="8"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="10"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="14"/>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7"/>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="14"/>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="7"/>
-    </row>
-    <row r="8" s="0" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="12"/>
-      <c r="B8" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="10"/>
-      <c r="E8"/>
-    </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="9"/>
+    </row>
+    <row r="9" s="0" customFormat="1" ht="15" customHeight="1">
+      <c r="A9" s="17"/>
       <c r="B9" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D9" s="10" t="s">
         <v>11</v>
       </c>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="14"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10"/>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="10"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11"/>
       <c r="B11" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="14"/>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="B12" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="B12" s="8"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="10"/>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13"/>
-      <c r="B13" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="7"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="14"/>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14"/>
-      <c r="B14" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="D14" s="10"/>
+      <c r="B14" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="16"/>
+      <c r="D14" s="16"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="9"/>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="B15" s="13"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="10"/>
+      <c r="B15" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="14"/>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="14"/>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="B17" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D17" s="10"/>
+      <c r="B17" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="20"/>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="B18" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="10"/>
+        <v>19</v>
+      </c>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F18" s="14"/>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="B19" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="10"/>
+        <v>20</v>
+      </c>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F19" s="14"/>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="B20" s="8"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="10"/>
+      <c r="B20" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="14"/>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="B21" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="C21" s="6"/>
-      <c r="D21" s="7"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="14"/>
     </row>
     <row r="22" ht="15" customHeight="1">
-      <c r="B22" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="18" t="s">
+      <c r="B22" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="9"/>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="B23" s="13" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="B23" s="8"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="10"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1">
-      <c r="B24" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="6"/>
-      <c r="D24" s="7"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="14"/>
     </row>
     <row r="25" ht="15" customHeight="1">
-      <c r="B25" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="19" t="s">
+      <c r="B25" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="9"/>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="B26" s="13" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="B26" s="8"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="10"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="14" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="B27" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="7"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="14"/>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="B28" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="10"/>
+      <c r="B28" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="F28" s="9"/>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="B29" s="8"/>
-      <c r="C29" s="21"/>
-      <c r="D29" s="10"/>
+      <c r="B29" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="F29" s="14"/>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="B30" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="7"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="14"/>
     </row>
     <row r="31" ht="15" customHeight="1">
-      <c r="B31" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="10" t="s">
+      <c r="B31" s="16" t="s">
         <v>32</v>
       </c>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="9"/>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="B32" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C32" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="10"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F32" s="14" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="B33" s="13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D33" s="10"/>
+        <v>35</v>
+      </c>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F33" s="14"/>
     </row>
     <row r="34" ht="15" customHeight="1">
       <c r="B34" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" s="10"/>
+        <v>36</v>
+      </c>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F34" s="14"/>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="B35" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" s="10"/>
+        <v>37</v>
+      </c>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F35" s="14"/>
     </row>
     <row r="36" ht="15" customHeight="1">
       <c r="B36" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="C36" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D36" s="10" t="s">
         <v>38</v>
       </c>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F36" s="14"/>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="B37" s="23" t="s">
+      <c r="B37" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C37" s="11"/>
-      <c r="D37" s="10"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F37" s="14" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="B38" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C38" s="6"/>
-      <c r="D38" s="7"/>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="B39" s="24" t="s">
+      <c r="B38" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C39" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D39" s="26" t="s">
+      <c r="C38" s="27"/>
+      <c r="D38" s="27"/>
+      <c r="E38" s="15"/>
+      <c r="F38" s="14"/>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="B39" s="16" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="40" ht="15" customHeight="1">
-      <c r="B40" s="13" t="s">
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="9"/>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="B40" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C40" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D40" s="10"/>
-    </row>
-    <row r="41" ht="27.75" customHeight="1">
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F40" s="30" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="41" ht="15" customHeight="1">
       <c r="B41" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C41" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="D41" s="28" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="42" ht="15" customHeight="1">
+      <c r="C41" s="13"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F41" s="14"/>
+    </row>
+    <row r="42" ht="27.75" customHeight="1">
       <c r="B42" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C42" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D42" s="10" t="s">
+      <c r="C42" s="13"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="F42" s="32" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
-      <c r="B43" s="8"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="10"/>
+      <c r="B43" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C43" s="13"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F43" s="14" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1">
-      <c r="B44" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C44" s="6"/>
-      <c r="D44" s="7"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="14"/>
     </row>
     <row r="45" ht="15" customHeight="1">
-      <c r="B45" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="C45" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D45" s="10"/>
+      <c r="B45" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="C45" s="16"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="9"/>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="B46" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="C46" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="D46" s="10"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F46" s="14"/>
     </row>
     <row r="47" ht="15" customHeight="1">
-      <c r="B47" s="8" t="s">
+      <c r="B47" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C47" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>47</v>
-      </c>
+      <c r="C47" s="13"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="F47" s="14"/>
     </row>
     <row r="48" ht="15" customHeight="1">
-      <c r="B48" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C48" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D48" s="10" t="s">
+      <c r="B48" s="13" t="s">
         <v>54</v>
       </c>
+      <c r="C48" s="13"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F48" s="14" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1">
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C49" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>54</v>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F49" s="14" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
-      <c r="B50" s="8" t="s">
+      <c r="B50" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C50" s="13"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F50" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C50" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D50" s="10" t="s">
-        <v>54</v>
-      </c>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="B51" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C51" s="22" t="s">
-        <v>5</v>
-      </c>
-      <c r="D51" s="10" t="s">
-        <v>47</v>
+      <c r="B51" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="13"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F51" s="14" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="B52" s="8"/>
-      <c r="C52" s="11"/>
-      <c r="D52" s="10"/>
+      <c r="B52" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="13"/>
+      <c r="D52" s="13"/>
+      <c r="E52" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F52" s="14" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1">
-      <c r="B53" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C53" s="6"/>
-      <c r="D53" s="7"/>
+      <c r="B53" s="13"/>
+      <c r="C53" s="13"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="15"/>
+      <c r="F53" s="14"/>
     </row>
     <row r="54" ht="15" customHeight="1">
-      <c r="B54" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D54" s="10"/>
+      <c r="B54" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C54" s="16"/>
+      <c r="D54" s="16"/>
+      <c r="E54" s="12"/>
+      <c r="F54" s="9"/>
     </row>
     <row r="55" ht="15" customHeight="1">
-      <c r="B55" s="8"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="10"/>
+      <c r="B55" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C55" s="1"/>
+      <c r="D55" s="1"/>
+      <c r="E55" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="F55" s="14"/>
     </row>
     <row r="56" ht="15" customHeight="1">
-      <c r="B56" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C56" s="6"/>
-      <c r="D56" s="7"/>
+      <c r="B56" s="13"/>
+      <c r="C56" s="13"/>
+      <c r="D56" s="13"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="14"/>
     </row>
     <row r="57" ht="15" customHeight="1">
-      <c r="B57" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C57" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="D57" s="10" t="s">
+      <c r="B57" s="16" t="s">
         <v>62</v>
       </c>
+      <c r="C57" s="16"/>
+      <c r="D57" s="16"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="9"/>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="B58" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C58" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="D58" s="10"/>
+      <c r="C58" s="13"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F58" s="14" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1">
-      <c r="B59" s="8"/>
-      <c r="C59" s="11"/>
-      <c r="D59" s="10"/>
+      <c r="B59" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C59" s="13"/>
+      <c r="D59" s="13"/>
+      <c r="E59" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F59" s="14"/>
     </row>
     <row r="60" ht="15" customHeight="1">
-      <c r="B60" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C60" s="6"/>
-      <c r="D60" s="7"/>
+      <c r="B60" s="13"/>
+      <c r="C60" s="13"/>
+      <c r="D60" s="13"/>
+      <c r="E60" s="15"/>
+      <c r="F60" s="14"/>
     </row>
     <row r="61" ht="15" customHeight="1">
-      <c r="B61" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="C61" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D61" s="10" t="s">
+      <c r="B61" s="16" t="s">
         <v>66</v>
       </c>
+      <c r="C61" s="16"/>
+      <c r="D61" s="16"/>
+      <c r="E61" s="12"/>
+      <c r="F61" s="9"/>
     </row>
     <row r="62" ht="15" customHeight="1">
-      <c r="B62" s="8" t="s">
+      <c r="B62" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="C62" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="D62" s="10"/>
+      <c r="C62" s="13"/>
+      <c r="D62" s="13"/>
+      <c r="E62" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F62" s="14" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="B63" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="C63" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D63" s="10"/>
+        <v>69</v>
+      </c>
+      <c r="C63" s="13"/>
+      <c r="D63" s="13"/>
+      <c r="E63" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="F63" s="14"/>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="B64" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="C64" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="D64" s="10" t="s">
         <v>70</v>
       </c>
+      <c r="C64" s="13"/>
+      <c r="D64" s="13"/>
+      <c r="E64" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F64" s="14"/>
     </row>
     <row r="65" ht="15" customHeight="1">
       <c r="B65" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="C65" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D65" s="10" t="s">
-        <v>70</v>
+      <c r="C65" s="13"/>
+      <c r="D65" s="13"/>
+      <c r="E65" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F65" s="14" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="B66" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C66" s="13"/>
+      <c r="D66" s="13"/>
+      <c r="E66" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F66" s="14" t="s">
         <v>72</v>
-      </c>
-      <c r="C66" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D66" s="10" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="B67" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C67" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D67" s="10" t="s">
         <v>74</v>
       </c>
+      <c r="C67" s="13"/>
+      <c r="D67" s="13"/>
+      <c r="E67" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F67" s="14" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="68" ht="15" customHeight="1">
-      <c r="B68" s="8"/>
-      <c r="C68" s="11"/>
-      <c r="D68" s="10"/>
+      <c r="B68" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="C68" s="13"/>
+      <c r="D68" s="13"/>
+      <c r="E68" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F68" s="14" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="69" ht="15" customHeight="1">
-      <c r="B69" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C69" s="6"/>
-      <c r="D69" s="7"/>
+      <c r="B69" s="13"/>
+      <c r="C69" s="13"/>
+      <c r="D69" s="13"/>
+      <c r="E69" s="15"/>
+      <c r="F69" s="14"/>
     </row>
     <row r="70" ht="15" customHeight="1">
-      <c r="B70" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="C70" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="D70" s="10"/>
+      <c r="B70" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C70" s="16"/>
+      <c r="D70" s="16"/>
+      <c r="E70" s="12"/>
+      <c r="F70" s="9"/>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="B71" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="C71" s="30" t="s">
-        <v>26</v>
-      </c>
-      <c r="D71" s="10"/>
+        <v>78</v>
+      </c>
+      <c r="C71" s="13"/>
+      <c r="D71" s="13"/>
+      <c r="E71" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F71" s="14"/>
     </row>
     <row r="72" ht="15" customHeight="1">
-      <c r="B72" s="8"/>
-      <c r="C72" s="11"/>
-      <c r="D72" s="10"/>
+      <c r="B72" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C72" s="13"/>
+      <c r="D72" s="13"/>
+      <c r="E72" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="F72" s="14"/>
     </row>
     <row r="73" ht="15" customHeight="1">
-      <c r="B73" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C73" s="6"/>
-      <c r="D73" s="7"/>
+      <c r="B73" s="13"/>
+      <c r="C73" s="13"/>
+      <c r="D73" s="13"/>
+      <c r="E73" s="15"/>
+      <c r="F73" s="14"/>
     </row>
     <row r="74" ht="15" customHeight="1">
-      <c r="B74" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="C74" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D74" s="10" t="s">
+      <c r="B74" s="16" t="s">
         <v>80</v>
       </c>
+      <c r="C74" s="16"/>
+      <c r="D74" s="16"/>
+      <c r="E74" s="12"/>
+      <c r="F74" s="9"/>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="B75" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="C75" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D75" s="10" t="s">
+      <c r="C75" s="13"/>
+      <c r="D75" s="13"/>
+      <c r="E75" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F75" s="14" t="s">
         <v>82</v>
       </c>
     </row>
@@ -2328,21 +2501,25 @@
       <c r="B76" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="C76" s="25" t="s">
-        <v>22</v>
-      </c>
-      <c r="D76" s="10" t="s">
+      <c r="C76" s="13"/>
+      <c r="D76" s="13"/>
+      <c r="E76" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F76" s="14" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
-      <c r="B77" s="8" t="s">
+      <c r="B77" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="C77" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D77" s="10" t="s">
+      <c r="C77" s="13"/>
+      <c r="D77" s="13"/>
+      <c r="E77" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F77" s="14" t="s">
         <v>86</v>
       </c>
     </row>
@@ -2350,118 +2527,141 @@
       <c r="B78" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="C78" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D78" s="10"/>
+      <c r="C78" s="13"/>
+      <c r="D78" s="13"/>
+      <c r="E78" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F78" s="14" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1">
       <c r="B79" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="C79" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="D79" s="10" t="s">
         <v>89</v>
       </c>
+      <c r="C79" s="13"/>
+      <c r="D79" s="13"/>
+      <c r="E79" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F79" s="14"/>
     </row>
     <row r="80" ht="15" customHeight="1">
-      <c r="B80" s="8"/>
-      <c r="C80" s="11"/>
-      <c r="D80" s="10"/>
+      <c r="B80" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C80" s="13"/>
+      <c r="D80" s="13"/>
+      <c r="E80" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="F80" s="14" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="81" ht="15" customHeight="1">
-      <c r="B81" s="1"/>
-      <c r="C81" s="2"/>
-      <c r="D81"/>
+      <c r="B81" s="13"/>
+      <c r="C81" s="13"/>
+      <c r="D81" s="13"/>
+      <c r="E81" s="15"/>
+      <c r="F81" s="14"/>
     </row>
     <row r="82" ht="15" customHeight="1">
       <c r="B82" s="1"/>
-      <c r="C82" s="2"/>
-      <c r="D82"/>
+      <c r="C82" s="1"/>
+      <c r="D82" s="1"/>
+      <c r="E82" s="2"/>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="B83" s="1"/>
-      <c r="C83" s="2"/>
-      <c r="D83"/>
+      <c r="C83" s="1"/>
+      <c r="D83" s="1"/>
+      <c r="E83" s="2"/>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="B84" s="1"/>
-      <c r="C84" s="2"/>
-      <c r="D84"/>
+      <c r="C84" s="1"/>
+      <c r="D84" s="1"/>
+      <c r="E84" s="2"/>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="B85" s="1"/>
-      <c r="C85" s="2"/>
-      <c r="D85"/>
+      <c r="C85" s="1"/>
+      <c r="D85" s="1"/>
+      <c r="E85" s="2"/>
     </row>
     <row r="86" ht="15" customHeight="1">
       <c r="B86" s="1"/>
-      <c r="C86" s="2"/>
-      <c r="D86"/>
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="2"/>
     </row>
     <row r="87" ht="15" customHeight="1">
       <c r="B87" s="1"/>
-      <c r="C87" s="2"/>
-      <c r="D87"/>
+      <c r="C87" s="1"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="2"/>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="B88" s="1"/>
-      <c r="C88" s="2"/>
-      <c r="D88"/>
+      <c r="C88" s="1"/>
+      <c r="D88" s="1"/>
+      <c r="E88" s="2"/>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="B89" s="1"/>
-      <c r="C89" s="2"/>
-      <c r="D89"/>
+      <c r="C89" s="1"/>
+      <c r="D89" s="1"/>
+      <c r="E89" s="2"/>
     </row>
     <row r="90" ht="15" customHeight="1">
       <c r="B90" s="1"/>
-      <c r="C90" s="2"/>
-      <c r="D90"/>
+      <c r="C90" s="1"/>
+      <c r="D90" s="1"/>
+      <c r="E90" s="2"/>
     </row>
     <row r="91" ht="15" customHeight="1">
       <c r="B91" s="1"/>
-      <c r="C91" s="2"/>
-      <c r="D91"/>
+      <c r="C91" s="1"/>
+      <c r="D91" s="1"/>
+      <c r="E91" s="2"/>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="B92" s="1"/>
-      <c r="C92" s="2"/>
-      <c r="D92"/>
+      <c r="C92" s="1"/>
+      <c r="D92" s="1"/>
+      <c r="E92" s="2"/>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="B93" s="1"/>
-      <c r="C93" s="2"/>
-      <c r="D93"/>
+      <c r="C93" s="1"/>
+      <c r="D93" s="1"/>
+      <c r="E93" s="2"/>
     </row>
     <row r="94" ht="15" customHeight="1">
       <c r="B94" s="1"/>
-      <c r="C94" s="2"/>
-      <c r="D94"/>
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="2"/>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="B95" s="1"/>
-      <c r="C95" s="2"/>
-      <c r="D95"/>
+      <c r="C95" s="1"/>
+      <c r="D95" s="1"/>
+      <c r="E95" s="2"/>
+    </row>
+    <row r="96" ht="15" customHeight="1">
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+      <c r="E96" s="2"/>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
-  </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" customHeight="1"/>
-  <sheetData/>
+  <mergeCells count="2">
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C3"/>
+  </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>

</xml_diff>